<commit_message>
fix(i18n): use natural English labels and licensing terminology
</commit_message>
<xml_diff>
--- a/vue-pure-admin/public/IP-import-template.en.xlsx
+++ b/vue-pure-admin/public/IP-import-template.en.xlsx
@@ -638,7 +638,7 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Contact person</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -663,12 +663,12 @@
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>Base rights price lower limit</t>
+          <t>Minimum licensing fee</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>Base rights price upper limit</t>
+          <t>Maximum licensing fee</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>IP image &amp; style</t>
+          <t>Visual identity and style</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
@@ -693,12 +693,12 @@
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>Primary age</t>
+          <t>Core age group</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
-          <t>Purchasing power assessment</t>
+          <t>Spending power</t>
         </is>
       </c>
       <c r="AJ1" s="1" t="inlineStr">
@@ -708,27 +708,27 @@
       </c>
       <c r="AK1" s="1" t="inlineStr">
         <is>
-          <t>Historical sales conversion strength</t>
+          <t>Past sales performance</t>
         </is>
       </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
-          <t>IP showcase &amp; collaboration performance</t>
+          <t>Portfolio and partnership results</t>
         </is>
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
-          <t>Collaboration recommendations &amp; reminders</t>
+          <t>Partnership recommendations and notes</t>
         </is>
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>Past collaboration name</t>
+          <t>Past partnership title</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>Past collaboration overview</t>
+          <t>Past partnership summary</t>
         </is>
       </c>
     </row>
@@ -22236,7 +22236,7 @@
   <autoFilter ref="A1:AO501"/>
   <dataValidations count="4">
     <dataValidation sqref="C2:C501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="请选择下拉选项" error="该字段请使用模板中的下拉选项。" promptTitle="IP type" prompt="请选择指定的IP类型。" type="list" errorStyle="stop">
-      <formula1>"Gaming,Animation,Film &amp; TV,Variety Shows,Sports,Streetwear,Designer Toys,Brands,Arts &amp; Culture,Offline Events,Other"</formula1>
+      <formula1>"Gaming,Animation,Film &amp; TV,Variety Shows,Sports,Streetwear,Designer Toys,Brands,Arts &amp; Culture,In-person events,Other"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D501 E2:E501 F2:F501 G2:G501 H2:H501 I2:I501 J2:J501 K2:K501 L2:L501" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Covered markets" prompt="每列选择一个市场；可使用多列。" type="list">
       <formula1>"China,Southeast Asia,South Asia,Europe,Middle East,Africa,Latin America,North America,Global"</formula1>
@@ -22287,7 +22287,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Choose a type from the dropdown: Gaming, Animation, Film &amp; TV, Variety Shows, Sports, Streetwear, Designer Toys, Brands, Arts &amp; Culture, Offline Events, Other.</t>
+          <t>Choose a type from the dropdown: Gaming, Animation, Film &amp; TV, Variety Shows, Sports, Streetwear, Designer Toys, Brands, Arts &amp; Culture, In-person events, Other.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ip): add collaboration format dropdowns to import templates
</commit_message>
<xml_diff>
--- a/vue-pure-admin/public/IP-import-template.en.xlsx
+++ b/vue-pure-admin/public/IP-import-template.en.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IP import" sheetId="1" r:id="Re508e2e255ad46cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rc3e8a6a9125444bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IP import" sheetId="1" r:id="Rc19c0ea6c3ba4c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Refb026f16e69475b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23240,7 +23240,7 @@
       <x:c r="AQ501" s="11"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="4">
+  <x:dataValidations count="5">
     <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="请选择下拉选项" error="该字段请使用模板中的下拉选项。" promptTitle="IP type" prompt="请选择指定的IP类型。" sqref="C2:C501">
       <x:formula1>"Gaming,Animation,Film &amp; TV,Variety Shows,Sports,Streetwear,Designer Toys,Brands,Arts &amp; Culture,In-person events,Other"</x:formula1>
     </x:dataValidation>
@@ -23254,9 +23254,12 @@
       <x:formula1>0</x:formula1>
       <x:formula2>100</x:formula2>
     </x:dataValidation>
+    <x:dataValidation type="list" allowBlank="1" showDropDown="0" showErrorMessage="0" sqref="AP2:AP501">
+      <x:formula1>"Product customization,Feature integration,Co-branded merchandise and gift boxes,Online marketing,Offline materials and activations"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38f01d0b8de24acf"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ac1580edb4546ea"/>
 </x:worksheet>
 </file>
 
@@ -23369,7 +23372,7 @@
         <x:v>Available collaboration formats</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>Optional. Separate multiple formats with / or ;. Options: Product customization; Feature integration; Co-branded merchandise and gift boxes; Online marketing; Offline materials and activations. Example: Product customization / Online marketing.</x:v>
+        <x:v>Optional. Choose one format from the dropdown. For multiple formats, type or paste options separated by / or ;. The dropdown replaces the cell value. Options: Product customization; Feature integration; Co-branded merchandise and gift boxes; Online marketing; Offline materials and activations.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="80" customHeight="1">

</xml_diff>